<commit_message>
V1.1 portable: signature, date field, RTL table, PDF/DOCX modes
Add V1.1 build/test scripts, output_format module, docx table builder, and updated templates. Include V1.2 audit report and performance data. Portable app.exe and ZIPs remain local (gitignored).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/תחשיב זכויות אישי/DB למכתב תחשיב זכויות וחובות.xlsx
+++ b/תחשיב זכויות אישי/DB למכתב תחשיב זכויות וחובות.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1SSJvtvpGqSvsTBfNxwKjp3PCgLcXP7lO\מענק 2026\מכתבים\מכתבי סכומים\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dfusb\Documents\מכונת מכתבים\תחשיב זכויות אישי\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A201FD6E-3CFD-4D63-8635-39DB6DA7D171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6B5EED-203E-4B00-80B8-CF576416478D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{230BCDDF-ECC3-443F-AB3B-8BCF8BF18170}"/>
+    <workbookView xWindow="2304" yWindow="972" windowWidth="17280" windowHeight="11988" xr2:uid="{230BCDDF-ECC3-443F-AB3B-8BCF8BF18170}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
   <si>
     <t>סידורי</t>
   </si>
@@ -132,6 +132,15 @@
   </si>
   <si>
     <t>חשבון בנק</t>
+  </si>
+  <si>
+    <t>12-34-5678</t>
+  </si>
+  <si>
+    <t>11-22-333</t>
+  </si>
+  <si>
+    <t>99-88-777</t>
   </si>
 </sst>
 </file>
@@ -139,13 +148,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="42" formatCode="_ &quot;₪&quot;\ * #,##0_ ;_ &quot;₪&quot;\ * \-#,##0_ ;_ &quot;₪&quot;\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;₪&quot;\ * #,##0_ ;_ &quot;₪&quot;\ * \-#,##0_ ;_ &quot;₪&quot;\ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -240,7 +249,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -267,7 +276,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -723,7 +732,9 @@
       <c r="R2" s="8">
         <v>132</v>
       </c>
-      <c r="S2" s="8"/>
+      <c r="S2" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="T2" s="8" t="s">
         <v>24</v>
       </c>
@@ -787,7 +798,9 @@
       </c>
       <c r="Q3" s="8"/>
       <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
+      <c r="S3" s="8" t="s">
+        <v>32</v>
+      </c>
       <c r="T3" s="8" t="s">
         <v>24</v>
       </c>
@@ -850,7 +863,9 @@
       </c>
       <c r="Q4" s="8"/>
       <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
+      <c r="S4" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="T4" s="8" t="s">
         <v>24</v>
       </c>

</xml_diff>